<commit_message>
feat(ui): 完成 FairyGUI 统一宿主接入
统一 FairyGUI 到 GF UIForm/UIGroup 宿主，补齐发布、描述符、绑定与资源规则。

保留可审计的 Trellis 设计与验证记录，并移除旧的每窗体 UIPanel POC。
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/Game/UI.xlsx
+++ b/Design/Excel/ET/Datas/Game/UI.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
-  <workbookPr/>
+  <workbookPr autoCompressPictures="1"/>
   <bookViews>
     <workbookView windowHeight="17800"/>
   </bookViews>
   <sheets>
     <sheet name="UI界面" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="0" refMode="A1" iterate="0" fullPrecision="0" calcCompleted="0" calcOnSave="0" concurrentCalc="0" forceFullCalc="0"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
+    <ext uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures">
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
@@ -27,168 +27,180 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="52">
-  <si>
-    <t>##var</t>
-  </si>
-  <si>
-    <t>Id</t>
-  </si>
-  <si>
-    <t>CSName</t>
-  </si>
-  <si>
-    <t>Desc</t>
-  </si>
-  <si>
-    <t>AssetName</t>
-  </si>
-  <si>
-    <t>UIGroupName</t>
-  </si>
-  <si>
-    <t>AllowMultiInstance</t>
-  </si>
-  <si>
-    <t>PauseCoveredUIForm</t>
-  </si>
-  <si>
-    <t>##type</t>
-  </si>
-  <si>
-    <t>int</t>
-  </si>
-  <si>
-    <t>string&amp;group=ge</t>
-  </si>
-  <si>
-    <t>string#path=normal;UI/UIForm/*.prefab</t>
-  </si>
-  <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>bool</t>
-  </si>
-  <si>
-    <t>##</t>
-  </si>
-  <si>
-    <t>界面编号</t>
-  </si>
-  <si>
-    <t>代码名（程序填）</t>
-  </si>
-  <si>
-    <t>备注</t>
-  </si>
-  <si>
-    <t>资源名称</t>
-  </si>
-  <si>
-    <t>界面组名称</t>
-  </si>
-  <si>
-    <t>是否允许多个界面实例</t>
-  </si>
-  <si>
-    <t>是否暂停被其覆盖的界面</t>
-  </si>
-  <si>
-    <t>UIHelp</t>
-  </si>
-  <si>
-    <t>帮助界面</t>
-  </si>
-  <si>
-    <t>Demo/UIHelp</t>
-  </si>
-  <si>
-    <t>Pop</t>
-  </si>
-  <si>
-    <t>UILobby</t>
-  </si>
-  <si>
-    <t>大厅面</t>
-  </si>
-  <si>
-    <t>Demo/UILobby</t>
-  </si>
-  <si>
-    <t>UILogin</t>
-  </si>
-  <si>
-    <t>登录界面</t>
-  </si>
-  <si>
-    <t>Demo/UILogin</t>
-  </si>
-  <si>
-    <t>Default</t>
-  </si>
-  <si>
-    <t>UILSLogin</t>
-  </si>
-  <si>
-    <t>LockStep/UILSLogin</t>
-  </si>
-  <si>
-    <t>UILSLobby</t>
-  </si>
-  <si>
-    <t>LockStep/UILSLobby</t>
-  </si>
-  <si>
-    <t>UILSRoom</t>
-  </si>
-  <si>
-    <t>房间界面</t>
-  </si>
-  <si>
-    <t>LockStep/UILSRoom</t>
-  </si>
-  <si>
-    <t>DialogForm</t>
-  </si>
-  <si>
-    <t>弹出框</t>
-  </si>
-  <si>
-    <t>Hot/DialogForm</t>
-  </si>
-  <si>
-    <t>MenuForm</t>
-  </si>
-  <si>
-    <t>主菜单</t>
-  </si>
-  <si>
-    <t>Hot/MenuForm</t>
-  </si>
-  <si>
-    <t>SettingForm</t>
-  </si>
-  <si>
-    <t>设置</t>
-  </si>
-  <si>
-    <t>Hot/SettingForm</t>
-  </si>
-  <si>
-    <t>AboutForm</t>
-  </si>
-  <si>
-    <t>关于</t>
-  </si>
-  <si>
-    <t>Hot/AboutForm</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="56">
+  <si>
+    <t xml:space="preserve">##var</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSName</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AssetName</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UIGroupName</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AllowMultiInstance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PauseCoveredUIForm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">##type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">int</t>
+  </si>
+  <si>
+    <t xml:space="preserve">string&amp;group=ge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">string#path=normal;UI/UIForm/*.prefab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">string</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">##</t>
+  </si>
+  <si>
+    <t xml:space="preserve">界面编号</t>
+  </si>
+  <si>
+    <t xml:space="preserve">代码名（程序填）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">备注</t>
+  </si>
+  <si>
+    <t xml:space="preserve">资源名称</t>
+  </si>
+  <si>
+    <t xml:space="preserve">界面组名称</t>
+  </si>
+  <si>
+    <t xml:space="preserve">是否允许多个界面实例</t>
+  </si>
+  <si>
+    <t xml:space="preserve">是否暂停被其覆盖的界面</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UIHelp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">帮助界面</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demo/UIHelp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UILobby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">大厅面</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demo/UILobby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UILogin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">登录界面</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demo/UILogin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Default</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UILSLogin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LockStep/UILSLogin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UILSLobby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LockStep/UILSLobby</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UILSRoom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">房间界面</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LockStep/UILSRoom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DialogForm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">弹出框</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hot/DialogForm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MenuForm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">主菜单</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hot/MenuForm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SettingForm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">设置</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hot/SettingForm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AboutForm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">关于</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hot/AboutForm</t>
+  </si>
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">FairyDemoForm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FairyGUI演示</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hot/FairyDemoForm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
@@ -204,26 +216,26 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <u val="single"/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
+      <charset/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u val="single"/>
       <sz val="11"/>
       <color rgb="FF800080"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -239,7 +251,7 @@
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -270,7 +282,7 @@
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -278,7 +290,7 @@
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -286,7 +298,7 @@
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -294,14 +306,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -309,42 +321,42 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C6500"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -650,154 +662,154 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" xfId="0" applyAlignment="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" xfId="0" applyAlignment="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -861,8 +873,8 @@
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1153,7 +1165,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr/>
   <dimension ref="A1:H13"/>
   <sheetFormatPr defaultColWidth="8.87272727272727" defaultRowHeight="14" outlineLevelCol="7"/>
@@ -1477,9 +1489,33 @@
         <v>1</v>
       </c>
     </row>
+    <row r="14">
+      <c r="B14" s="3">
+        <v>103</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G14" s="3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H14" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
+  <sheetCalcPr fullCalcOnLoad="1"/>
   <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(fgui): 新增 RuntimeInspector 界面与双端 Presenter
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/Game/UI.xlsx
+++ b/Design/Excel/ET/Datas/Game/UI.xlsx
@@ -1027,7 +1027,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.872727272727269" defaultRowHeight="14"/>
   <cols>
     <col width="8.872727272727269" customWidth="1" style="3" min="1" max="1"/>
@@ -1361,6 +1361,47 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="B8" t="n">
+        <v>107</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>FairyRuntimeInspectorForm</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>运行时调试面板</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>FairyGUI/FairyRuntimeInspectorForm</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>RuntimeInspector</t>
+        </is>
+      </c>
+      <c r="G8" t="b">
+        <v>0</v>
+      </c>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Package1</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>RuntimeInspectorView</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0"/>

</xml_diff>

<commit_message>
feat(fairygui): UI 表加 FullScreen 列并清空 WidgetTest 悬空实体
- UI.xlsx(GameHot+ET)加 FullScreen 列,106 InventoryOverlayForm 标记 true。
- 清空 UIEntity.xlsx 的 WidgetTest 悬空实体(prefab 已删,导致 Luban PathValidator 失败)。
- Luban 导出:DRUIForm 加 FullScreen 字段,dtuiform 数据 106=true。
- 重新生成 descriptor:FairyInventoryOverlayForm fullScreen=true,其余 false。
</commit_message>
<xml_diff>
--- a/Design/Excel/ET/Datas/Game/UI.xlsx
+++ b/Design/Excel/ET/Datas/Game/UI.xlsx
@@ -1,16 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr autoCompressPictures="1"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowHeight="17800" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView windowHeight="17800" tabRatio="600"/>
   </bookViews>
   <sheets>
-    <sheet name="UI界面" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="UI界面" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="0" refMode="A1" iterate="0" fullPrecision="0" calcCompleted="0" calcOnSave="0" concurrentCalc="0" forceFullCalc="0"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="4">
+  <si>
+    <t xml:space="preserve"/>
+  </si>
+  <si>
+    <t xml:space="preserve">FullScreen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bool</t>
+  </si>
+  <si>
+    <t xml:space="preserve">是否全屏</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -18,145 +34,145 @@
   <numFmts count="0"/>
   <fonts count="20">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FF800080"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FFFF0000"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="18"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <i val="1"/>
-      <color rgb="FF7F7F7F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="15"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="13"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="3"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FF3F3F76"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <b val="1"/>
-      <color rgb="FF3F3F3F"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <b val="1"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <b val="1"/>
-      <color rgb="FFFFFFFF"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FFFA7D00"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <b val="1"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FF006100"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FF9C0006"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color rgb="FF9C6500"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color theme="0"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="宋体"/>
-      <color theme="1"/>
-      <sz val="11"/>
+      <name val="宋体"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -456,161 +472,161 @@
     </border>
   </borders>
   <cellStyleXfs count="49">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1022,203 +1038,212 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J8"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.872727272727269" defaultRowHeight="14"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.87272727272727" defaultRowHeight="14"/>
   <cols>
-    <col width="8.872727272727269" customWidth="1" style="3" min="1" max="1"/>
-    <col width="19.3727272727273" customWidth="1" style="3" min="2" max="2"/>
-    <col width="20.7545454545455" customWidth="1" style="3" min="3" max="3"/>
-    <col width="22" customWidth="1" style="3" min="4" max="4"/>
-    <col width="52.1818181818182" customWidth="1" style="3" min="5" max="5"/>
-    <col width="14.6272727272727" customWidth="1" style="3" min="6" max="6"/>
-    <col width="23.1272727272727" customWidth="1" style="3" min="7" max="7"/>
-    <col width="23" customWidth="1" style="3" min="8" max="8"/>
-    <col width="8.872727272727269" customWidth="1" style="3" min="9" max="16384"/>
+    <col min="1" max="1" width="8.87272727272727" style="3" customWidth="1"/>
+    <col min="2" max="2" width="19.3727272727273" style="3" customWidth="1"/>
+    <col min="3" max="3" width="20.7545454545455" style="3" customWidth="1"/>
+    <col min="4" max="4" width="22" style="3" customWidth="1"/>
+    <col min="5" max="5" width="52.1818181818182" style="3" customWidth="1"/>
+    <col min="6" max="6" width="14.6272727272727" style="3" customWidth="1"/>
+    <col min="7" max="7" width="23.1272727272727" style="3" customWidth="1"/>
+    <col min="8" max="8" width="23" style="3" customWidth="1"/>
+    <col min="9" max="16384" width="8.87272727272727" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>##var</t>
+          <t xml:space="preserve">##var</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Id</t>
+          <t xml:space="preserve">Id</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>CSName</t>
+          <t xml:space="preserve">CSName</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Desc</t>
+          <t xml:space="preserve">Desc</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>AssetName</t>
+          <t xml:space="preserve">AssetName</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>UIGroupName</t>
+          <t xml:space="preserve">UIGroupName</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
         <is>
-          <t>AllowMultiInstance</t>
+          <t xml:space="preserve">AllowMultiInstance</t>
         </is>
       </c>
       <c r="H1" s="3" t="inlineStr">
         <is>
-          <t>PauseCoveredUIForm</t>
+          <t xml:space="preserve">PauseCoveredUIForm</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>PackageName</t>
+          <t xml:space="preserve">PackageName</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>ComponentName</t>
-        </is>
+          <t xml:space="preserve">ComponentName</t>
+        </is>
+      </c>
+      <c r="K1" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>##type</t>
+          <t xml:space="preserve">##type</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>int</t>
+          <t xml:space="preserve">int</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>string&amp;group=ge</t>
+          <t xml:space="preserve">string&amp;group=ge</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>string&amp;group=ge</t>
+          <t xml:space="preserve">string&amp;group=ge</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>string#path=normalAny;UI/*.json</t>
+          <t xml:space="preserve">string#path=normalAny;UI/*.json</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t xml:space="preserve">string</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t xml:space="preserve">bool</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t xml:space="preserve">string</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>string</t>
-        </is>
+          <t xml:space="preserve">string</t>
+        </is>
+      </c>
+      <c r="K2" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>##</t>
+          <t xml:space="preserve">##</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>界面编号</t>
+          <t xml:space="preserve">界面编号</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>代码名（程序填）</t>
+          <t xml:space="preserve">代码名（程序填）</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t xml:space="preserve">备注</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>资源名称</t>
+          <t xml:space="preserve">资源名称</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>界面组名称</t>
+          <t xml:space="preserve">界面组名称</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>是否允许多个界面实例</t>
+          <t xml:space="preserve">是否允许多个界面实例</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>是否暂停被其覆盖的界面</t>
+          <t xml:space="preserve">是否暂停被其覆盖的界面</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>包名</t>
+          <t xml:space="preserve">包名</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>组件名</t>
-        </is>
+          <t xml:space="preserve">组件名</t>
+        </is>
+      </c>
+      <c r="K3" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="3">
         <v>103</v>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>FairyDemoForm</t>
+          <t xml:space="preserve">FairyDemoForm</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI演示</t>
+          <t xml:space="preserve">FairyGUI演示</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI/FairyDemoForm</t>
+          <t xml:space="preserve">FairyGUI/FairyDemoForm</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t xml:space="preserve">Default</t>
         </is>
       </c>
       <c r="G4" s="3" t="b">
@@ -1229,37 +1254,40 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Package1</t>
+          <t xml:space="preserve">Package1</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>MainView</t>
-        </is>
+          <t xml:space="preserve">MainView</t>
+        </is>
+      </c>
+      <c r="K4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="3">
         <v>104</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>FairyInventoryForm</t>
+          <t xml:space="preserve">FairyInventoryForm</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI背包界面</t>
+          <t xml:space="preserve">FairyGUI背包界面</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI/FairyInventoryForm</t>
+          <t xml:space="preserve">FairyGUI/FairyInventoryForm</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t xml:space="preserve">Default</t>
         </is>
       </c>
       <c r="G5" s="3" t="b">
@@ -1270,37 +1298,40 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Package1</t>
+          <t xml:space="preserve">Package1</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>InventoryView</t>
-        </is>
+          <t xml:space="preserve">InventoryView</t>
+        </is>
+      </c>
+      <c r="K5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="3">
         <v>105</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>FairyItemDetailForm</t>
+          <t xml:space="preserve">FairyItemDetailForm</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI物品详情浮动窗口</t>
+          <t xml:space="preserve">FairyGUI物品详情浮动窗口</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI/FairyItemDetailForm</t>
+          <t xml:space="preserve">FairyGUI/FairyItemDetailForm</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Pop</t>
+          <t xml:space="preserve">Pop</t>
         </is>
       </c>
       <c r="G6" s="3" t="b">
@@ -1311,37 +1342,40 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Package1</t>
+          <t xml:space="preserve">Package1</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>ItemDetailWindow</t>
-        </is>
+          <t xml:space="preserve">ItemDetailWindow</t>
+        </is>
+      </c>
+      <c r="K6" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="3">
         <v>106</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>FairyInventoryOverlayForm</t>
+          <t xml:space="preserve">FairyInventoryOverlayForm</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI背包遮罩界面</t>
+          <t xml:space="preserve">FairyGUI背包遮罩界面</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>FairyGUI/FairyInventoryOverlayForm</t>
+          <t xml:space="preserve">FairyGUI/FairyInventoryOverlayForm</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Pop</t>
+          <t xml:space="preserve">Pop</t>
         </is>
       </c>
       <c r="G7" s="3" t="b">
@@ -1352,37 +1386,40 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Package1</t>
+          <t xml:space="preserve">Package1</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>InventoryOverlayView</t>
-        </is>
+          <t xml:space="preserve">InventoryOverlayView</t>
+        </is>
+      </c>
+      <c r="K7" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" t="n">
+      <c r="B8">
         <v>107</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>FairyRuntimeInspectorForm</t>
+          <t xml:space="preserve">FairyRuntimeInspectorForm</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>运行时调试面板</t>
+          <t xml:space="preserve">运行时调试面板</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>FairyGUI/FairyRuntimeInspectorForm</t>
+          <t xml:space="preserve">FairyGUI/FairyRuntimeInspectorForm</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>RuntimeInspector</t>
+          <t xml:space="preserve">RuntimeInspector</t>
         </is>
       </c>
       <c r="G8" t="b">
@@ -1393,17 +1430,21 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Package1</t>
+          <t xml:space="preserve">Package1</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>RuntimeInspectorView</t>
-        </is>
+          <t xml:space="preserve">RuntimeInspectorView</t>
+        </is>
+      </c>
+      <c r="K8" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
+  <sheetCalcPr fullCalcOnLoad="1"/>
   <pageMargins left="0.699305555555556" right="0.699305555555556" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>